<commit_message>
updated the total file
</commit_message>
<xml_diff>
--- a/dataset/total_data_excel.xlsx
+++ b/dataset/total_data_excel.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ulcampus-my.sharepoint.com/personal/toheeb_jimoh_ul_ie/Documents/SFI CRT DATA SCIENCE/Research Work/sarcasm_detection_LRL/Writings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_4F498382974C360F62355476585DCE3A87570A73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{914ED551-781E-F141-826D-82AFB98E7123}"/>
+  <xr:revisionPtr revIDLastSave="118" documentId="11_4F498382974C360F62355476585DCE3A87570A73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{708CDBB8-F786-2842-B7E8-3CF1B822E8A0}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9001" uniqueCount="4490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9202" uniqueCount="4491">
   <si>
     <t>S/N</t>
   </si>
@@ -13524,6 +13537,9 @@
   </si>
   <si>
     <t>The authors propose extending the dataset with contextual information or sarcasm-type labels to better guide models, and explore incorporating heterogeneous models into ensembles or Mixture-of-Experts (MoE) approaches with sub-models focusing on different aspects of sarcasm.</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -13600,6 +13616,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -14313,9 +14333,15 @@
       <c r="AT2" t="s">
         <v>135</v>
       </c>
+      <c r="AU2" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV2" t="s">
         <v>135</v>
       </c>
+      <c r="AW2" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX2" t="s">
         <v>136</v>
       </c>
@@ -14369,6 +14395,9 @@
       </c>
       <c r="BP2" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ2" t="s">
+        <v>128</v>
       </c>
       <c r="BR2" t="s">
         <v>108</v>
@@ -14857,8 +14886,14 @@
       <c r="AT4" t="s">
         <v>135</v>
       </c>
+      <c r="AU4" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV4" t="s">
         <v>135</v>
+      </c>
+      <c r="AW4" t="s">
+        <v>4490</v>
       </c>
       <c r="AX4" t="s">
         <v>241</v>
@@ -15132,8 +15167,14 @@
       <c r="AT5" t="s">
         <v>135</v>
       </c>
+      <c r="AU5" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV5" t="s">
         <v>135</v>
+      </c>
+      <c r="AW5" t="s">
+        <v>4490</v>
       </c>
       <c r="AX5" t="s">
         <v>282</v>
@@ -15335,6 +15376,9 @@
       <c r="U6" t="s">
         <v>135</v>
       </c>
+      <c r="V6" t="s">
+        <v>4490</v>
+      </c>
       <c r="W6" t="s">
         <v>313</v>
       </c>
@@ -15409,6 +15453,9 @@
       </c>
       <c r="AV6" t="s">
         <v>135</v>
+      </c>
+      <c r="AW6" t="s">
+        <v>4490</v>
       </c>
       <c r="AX6" t="s">
         <v>324</v>
@@ -15610,6 +15657,9 @@
       <c r="U7" t="s">
         <v>135</v>
       </c>
+      <c r="V7" t="s">
+        <v>4490</v>
+      </c>
       <c r="W7" t="s">
         <v>360</v>
       </c>
@@ -15744,6 +15794,9 @@
       </c>
       <c r="BP7" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ7" t="s">
+        <v>128</v>
       </c>
       <c r="BR7" t="s">
         <v>108</v>
@@ -15954,8 +16007,14 @@
       <c r="AT8" t="s">
         <v>135</v>
       </c>
+      <c r="AU8" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV8" t="s">
         <v>135</v>
+      </c>
+      <c r="AW8" t="s">
+        <v>4490</v>
       </c>
       <c r="AX8" t="s">
         <v>412</v>
@@ -16157,6 +16216,9 @@
       <c r="U9" t="s">
         <v>135</v>
       </c>
+      <c r="V9" t="s">
+        <v>4490</v>
+      </c>
       <c r="W9" t="s">
         <v>446</v>
       </c>
@@ -16229,6 +16291,9 @@
       <c r="AT9" t="s">
         <v>135</v>
       </c>
+      <c r="AU9" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV9" t="s">
         <v>193</v>
       </c>
@@ -16291,6 +16356,9 @@
       </c>
       <c r="BP9" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ9" t="s">
+        <v>128</v>
       </c>
       <c r="BR9" t="s">
         <v>108</v>
@@ -16429,6 +16497,9 @@
       <c r="U10" t="s">
         <v>135</v>
       </c>
+      <c r="V10" t="s">
+        <v>4490</v>
+      </c>
       <c r="W10" t="s">
         <v>487</v>
       </c>
@@ -16707,6 +16778,9 @@
       <c r="U11" t="s">
         <v>135</v>
       </c>
+      <c r="V11" t="s">
+        <v>4490</v>
+      </c>
       <c r="W11" t="s">
         <v>535</v>
       </c>
@@ -16776,8 +16850,14 @@
       <c r="AT11" t="s">
         <v>135</v>
       </c>
+      <c r="AU11" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV11" t="s">
         <v>135</v>
+      </c>
+      <c r="AW11" t="s">
+        <v>4490</v>
       </c>
       <c r="AX11" t="s">
         <v>543</v>
@@ -16973,6 +17053,9 @@
       <c r="U12" t="s">
         <v>135</v>
       </c>
+      <c r="V12" t="s">
+        <v>4490</v>
+      </c>
       <c r="W12" t="s">
         <v>573</v>
       </c>
@@ -17045,6 +17128,9 @@
       <c r="AT12" t="s">
         <v>135</v>
       </c>
+      <c r="AU12" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV12" t="s">
         <v>193</v>
       </c>
@@ -17107,6 +17193,9 @@
       </c>
       <c r="BP12" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ12" t="s">
+        <v>128</v>
       </c>
       <c r="BR12" t="s">
         <v>600</v>
@@ -17251,6 +17340,9 @@
       <c r="U13" t="s">
         <v>135</v>
       </c>
+      <c r="V13" t="s">
+        <v>4490</v>
+      </c>
       <c r="W13" t="s">
         <v>625</v>
       </c>
@@ -17328,6 +17420,9 @@
       </c>
       <c r="AV13" t="s">
         <v>135</v>
+      </c>
+      <c r="AW13" t="s">
+        <v>4490</v>
       </c>
       <c r="AX13" t="s">
         <v>638</v>
@@ -17529,6 +17624,9 @@
       <c r="U14" t="s">
         <v>135</v>
       </c>
+      <c r="V14" t="s">
+        <v>4490</v>
+      </c>
       <c r="W14" t="s">
         <v>672</v>
       </c>
@@ -17604,6 +17702,9 @@
       <c r="AV14" t="s">
         <v>135</v>
       </c>
+      <c r="AW14" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX14" t="s">
         <v>687</v>
       </c>
@@ -17660,6 +17761,9 @@
       </c>
       <c r="BP14" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ14" t="s">
+        <v>128</v>
       </c>
       <c r="BR14" t="s">
         <v>108</v>
@@ -17876,6 +17980,9 @@
       <c r="AV15" t="s">
         <v>135</v>
       </c>
+      <c r="AW15" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX15" t="s">
         <v>725</v>
       </c>
@@ -17929,6 +18036,9 @@
       </c>
       <c r="BP15" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ15" t="s">
+        <v>128</v>
       </c>
       <c r="BR15" t="s">
         <v>108</v>
@@ -18067,6 +18177,9 @@
       <c r="U16" t="s">
         <v>135</v>
       </c>
+      <c r="V16" t="s">
+        <v>4490</v>
+      </c>
       <c r="W16" t="s">
         <v>751</v>
       </c>
@@ -18142,6 +18255,9 @@
       <c r="AV16" t="s">
         <v>108</v>
       </c>
+      <c r="AW16" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX16" t="s">
         <v>371</v>
       </c>
@@ -18198,6 +18314,9 @@
       </c>
       <c r="BP16" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ16" t="s">
+        <v>128</v>
       </c>
       <c r="BR16" t="s">
         <v>108</v>
@@ -18420,6 +18539,9 @@
       <c r="AV17" t="s">
         <v>135</v>
       </c>
+      <c r="AW17" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX17" t="s">
         <v>809</v>
       </c>
@@ -18620,6 +18742,9 @@
       <c r="U18" t="s">
         <v>135</v>
       </c>
+      <c r="V18" t="s">
+        <v>4490</v>
+      </c>
       <c r="W18" t="s">
         <v>845</v>
       </c>
@@ -18691,6 +18816,9 @@
       </c>
       <c r="AT18" t="s">
         <v>135</v>
+      </c>
+      <c r="AU18" t="s">
+        <v>4490</v>
       </c>
       <c r="AV18" t="s">
         <v>193</v>
@@ -18973,8 +19101,14 @@
       <c r="AT19" t="s">
         <v>135</v>
       </c>
+      <c r="AU19" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV19" t="s">
         <v>135</v>
+      </c>
+      <c r="AW19" t="s">
+        <v>4490</v>
       </c>
       <c r="AX19" t="s">
         <v>918</v>
@@ -19176,6 +19310,9 @@
       <c r="U20" t="s">
         <v>135</v>
       </c>
+      <c r="V20" t="s">
+        <v>4490</v>
+      </c>
       <c r="W20" t="s">
         <v>956</v>
       </c>
@@ -19253,6 +19390,9 @@
       </c>
       <c r="AV20" t="s">
         <v>135</v>
+      </c>
+      <c r="AW20" t="s">
+        <v>4490</v>
       </c>
       <c r="AX20" t="s">
         <v>968</v>
@@ -19451,6 +19591,9 @@
       <c r="U21" t="s">
         <v>135</v>
       </c>
+      <c r="V21" t="s">
+        <v>4490</v>
+      </c>
       <c r="W21" t="s">
         <v>1002</v>
       </c>
@@ -19723,6 +19866,9 @@
       <c r="U22" t="s">
         <v>135</v>
       </c>
+      <c r="V22" t="s">
+        <v>4490</v>
+      </c>
       <c r="W22" t="s">
         <v>1058</v>
       </c>
@@ -19800,6 +19946,9 @@
       </c>
       <c r="AV22" t="s">
         <v>135</v>
+      </c>
+      <c r="AW22" t="s">
+        <v>4490</v>
       </c>
       <c r="AX22" t="s">
         <v>1080</v>
@@ -20004,6 +20153,9 @@
       <c r="U23" t="s">
         <v>135</v>
       </c>
+      <c r="V23" t="s">
+        <v>4490</v>
+      </c>
       <c r="W23" t="s">
         <v>1128</v>
       </c>
@@ -20135,6 +20287,9 @@
       </c>
       <c r="BP23" t="s">
         <v>1156</v>
+      </c>
+      <c r="BQ23" t="s">
+        <v>128</v>
       </c>
       <c r="BR23" t="s">
         <v>108</v>
@@ -20557,6 +20712,9 @@
       <c r="U25" t="s">
         <v>135</v>
       </c>
+      <c r="V25" t="s">
+        <v>4490</v>
+      </c>
       <c r="W25" t="s">
         <v>1238</v>
       </c>
@@ -20622,6 +20780,9 @@
       </c>
       <c r="AT25" t="s">
         <v>135</v>
+      </c>
+      <c r="AU25" t="s">
+        <v>4490</v>
       </c>
       <c r="AV25" t="s">
         <v>1250</v>
@@ -20823,6 +20984,9 @@
       <c r="U26" t="s">
         <v>135</v>
       </c>
+      <c r="V26" t="s">
+        <v>4490</v>
+      </c>
       <c r="W26" t="s">
         <v>1288</v>
       </c>
@@ -21095,6 +21259,9 @@
       <c r="U27" t="s">
         <v>135</v>
       </c>
+      <c r="V27" t="s">
+        <v>4490</v>
+      </c>
       <c r="W27" t="s">
         <v>1346</v>
       </c>
@@ -21170,6 +21337,9 @@
       <c r="AV27" t="s">
         <v>135</v>
       </c>
+      <c r="AW27" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX27" t="s">
         <v>371</v>
       </c>
@@ -21223,6 +21393,9 @@
       </c>
       <c r="BP27" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ27" t="s">
+        <v>128</v>
       </c>
       <c r="BR27" t="s">
         <v>108</v>
@@ -21448,6 +21621,9 @@
       <c r="AV28" t="s">
         <v>135</v>
       </c>
+      <c r="AW28" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX28" t="s">
         <v>371</v>
       </c>
@@ -21783,6 +21959,9 @@
       <c r="BP29" t="s">
         <v>135</v>
       </c>
+      <c r="BQ29" t="s">
+        <v>128</v>
+      </c>
       <c r="BR29" t="s">
         <v>108</v>
       </c>
@@ -21926,6 +22105,9 @@
       <c r="U30" t="s">
         <v>135</v>
       </c>
+      <c r="V30" t="s">
+        <v>4490</v>
+      </c>
       <c r="W30" t="s">
         <v>1489</v>
       </c>
@@ -22000,6 +22182,9 @@
       </c>
       <c r="AV30" t="s">
         <v>135</v>
+      </c>
+      <c r="AW30" t="s">
+        <v>4490</v>
       </c>
       <c r="AX30" t="s">
         <v>371</v>
@@ -22201,6 +22386,9 @@
       <c r="U31" t="s">
         <v>135</v>
       </c>
+      <c r="V31" t="s">
+        <v>4490</v>
+      </c>
       <c r="W31" t="s">
         <v>1533</v>
       </c>
@@ -22479,6 +22667,9 @@
       <c r="U32" t="s">
         <v>135</v>
       </c>
+      <c r="V32" t="s">
+        <v>4490</v>
+      </c>
       <c r="W32" t="s">
         <v>1580</v>
       </c>
@@ -22835,6 +23026,9 @@
       <c r="AV33" t="s">
         <v>135</v>
       </c>
+      <c r="AW33" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX33" t="s">
         <v>371</v>
       </c>
@@ -23035,6 +23229,9 @@
       <c r="U34" t="s">
         <v>135</v>
       </c>
+      <c r="V34" t="s">
+        <v>4490</v>
+      </c>
       <c r="W34" t="s">
         <v>1662</v>
       </c>
@@ -23104,6 +23301,9 @@
       <c r="AT34" t="s">
         <v>135</v>
       </c>
+      <c r="AU34" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV34" t="s">
         <v>193</v>
       </c>
@@ -23163,6 +23363,9 @@
       </c>
       <c r="BP34" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ34" t="s">
+        <v>128</v>
       </c>
       <c r="BR34" t="s">
         <v>108</v>
@@ -23307,6 +23510,9 @@
       <c r="U35" t="s">
         <v>135</v>
       </c>
+      <c r="V35" t="s">
+        <v>4490</v>
+      </c>
       <c r="W35" t="s">
         <v>1701</v>
       </c>
@@ -23376,9 +23582,15 @@
       <c r="AT35" t="s">
         <v>135</v>
       </c>
+      <c r="AU35" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV35" t="s">
         <v>135</v>
       </c>
+      <c r="AW35" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX35" t="s">
         <v>1713</v>
       </c>
@@ -23432,6 +23644,9 @@
       </c>
       <c r="BP35" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ35" t="s">
+        <v>128</v>
       </c>
       <c r="BR35" t="s">
         <v>108</v>
@@ -23576,6 +23791,9 @@
       <c r="U36" t="s">
         <v>135</v>
       </c>
+      <c r="V36" t="s">
+        <v>4490</v>
+      </c>
       <c r="W36" t="s">
         <v>1742</v>
       </c>
@@ -23645,6 +23863,9 @@
       <c r="AT36" t="s">
         <v>135</v>
       </c>
+      <c r="AU36" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV36" t="s">
         <v>193</v>
       </c>
@@ -23704,6 +23925,9 @@
       </c>
       <c r="BP36" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ36" t="s">
+        <v>128</v>
       </c>
       <c r="BR36" t="s">
         <v>108</v>
@@ -23848,6 +24072,9 @@
       <c r="U37" t="s">
         <v>135</v>
       </c>
+      <c r="V37" t="s">
+        <v>4490</v>
+      </c>
       <c r="W37" t="s">
         <v>1782</v>
       </c>
@@ -23925,6 +24152,9 @@
       </c>
       <c r="AV37" t="s">
         <v>135</v>
+      </c>
+      <c r="AW37" t="s">
+        <v>4490</v>
       </c>
       <c r="AX37" t="s">
         <v>1796</v>
@@ -24261,6 +24491,9 @@
       <c r="BP38" t="s">
         <v>135</v>
       </c>
+      <c r="BQ38" t="s">
+        <v>128</v>
+      </c>
       <c r="BR38" t="s">
         <v>108</v>
       </c>
@@ -24482,6 +24715,9 @@
       <c r="AV39" t="s">
         <v>135</v>
       </c>
+      <c r="AW39" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX39" t="s">
         <v>371</v>
       </c>
@@ -24676,6 +24912,9 @@
       <c r="U40" t="s">
         <v>135</v>
       </c>
+      <c r="V40" t="s">
+        <v>4490</v>
+      </c>
       <c r="W40" t="s">
         <v>1912</v>
       </c>
@@ -24807,6 +25046,9 @@
       </c>
       <c r="BP40" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ40" t="s">
+        <v>128</v>
       </c>
       <c r="BR40" t="s">
         <v>108</v>
@@ -24951,6 +25193,9 @@
       <c r="U41" t="s">
         <v>135</v>
       </c>
+      <c r="V41" t="s">
+        <v>4490</v>
+      </c>
       <c r="W41" t="s">
         <v>1942</v>
       </c>
@@ -25020,8 +25265,14 @@
       <c r="AT41" t="s">
         <v>135</v>
       </c>
+      <c r="AU41" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV41" t="s">
         <v>135</v>
+      </c>
+      <c r="AW41" t="s">
+        <v>4490</v>
       </c>
       <c r="AX41" t="s">
         <v>1950</v>
@@ -25223,6 +25474,9 @@
       <c r="U42" t="s">
         <v>135</v>
       </c>
+      <c r="V42" t="s">
+        <v>4490</v>
+      </c>
       <c r="W42" t="s">
         <v>1981</v>
       </c>
@@ -25582,6 +25836,9 @@
       <c r="AV43" t="s">
         <v>135</v>
       </c>
+      <c r="AW43" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX43" t="s">
         <v>2033</v>
       </c>
@@ -25854,6 +26111,9 @@
       <c r="AV44" t="s">
         <v>135</v>
       </c>
+      <c r="AW44" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX44" t="s">
         <v>2073</v>
       </c>
@@ -25910,6 +26170,9 @@
       </c>
       <c r="BP44" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ44" t="s">
+        <v>128</v>
       </c>
       <c r="BR44" t="s">
         <v>108</v>
@@ -26132,6 +26395,9 @@
       <c r="AV45" t="s">
         <v>135</v>
       </c>
+      <c r="AW45" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX45" t="s">
         <v>2102</v>
       </c>
@@ -26185,6 +26451,9 @@
       </c>
       <c r="BP45" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ45" t="s">
+        <v>128</v>
       </c>
       <c r="BR45" t="s">
         <v>1958</v>
@@ -26407,6 +26676,9 @@
       <c r="AV46" t="s">
         <v>135</v>
       </c>
+      <c r="AW46" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX46" t="s">
         <v>2128</v>
       </c>
@@ -26954,8 +27226,14 @@
       <c r="AT48" t="s">
         <v>135</v>
       </c>
+      <c r="AU48" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV48" t="s">
         <v>135</v>
+      </c>
+      <c r="AW48" t="s">
+        <v>4490</v>
       </c>
       <c r="AX48" t="s">
         <v>2213</v>
@@ -27235,6 +27513,9 @@
       <c r="AV49" t="s">
         <v>135</v>
       </c>
+      <c r="AW49" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX49" t="s">
         <v>2245</v>
       </c>
@@ -27507,8 +27788,14 @@
       <c r="AT50" t="s">
         <v>135</v>
       </c>
+      <c r="AU50" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV50" t="s">
         <v>135</v>
+      </c>
+      <c r="AW50" t="s">
+        <v>4490</v>
       </c>
       <c r="AX50" t="s">
         <v>2274</v>
@@ -27704,6 +27991,9 @@
       <c r="U51" t="s">
         <v>135</v>
       </c>
+      <c r="V51" t="s">
+        <v>4490</v>
+      </c>
       <c r="W51" t="s">
         <v>2294</v>
       </c>
@@ -27775,6 +28065,9 @@
       </c>
       <c r="AT51" t="s">
         <v>135</v>
+      </c>
+      <c r="AU51" t="s">
+        <v>4490</v>
       </c>
       <c r="AV51" t="s">
         <v>193</v>
@@ -27985,6 +28278,9 @@
       <c r="U52" t="s">
         <v>135</v>
       </c>
+      <c r="V52" t="s">
+        <v>4490</v>
+      </c>
       <c r="W52" t="s">
         <v>2328</v>
       </c>
@@ -28341,6 +28637,9 @@
       <c r="AV53" t="s">
         <v>135</v>
       </c>
+      <c r="AW53" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX53" t="s">
         <v>2371</v>
       </c>
@@ -28541,6 +28840,9 @@
       <c r="U54" t="s">
         <v>135</v>
       </c>
+      <c r="V54" t="s">
+        <v>4490</v>
+      </c>
       <c r="W54" t="s">
         <v>2398</v>
       </c>
@@ -28610,8 +28912,14 @@
       <c r="AT54" t="s">
         <v>135</v>
       </c>
+      <c r="AU54" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV54" t="s">
         <v>135</v>
+      </c>
+      <c r="AW54" t="s">
+        <v>4490</v>
       </c>
       <c r="AX54" t="s">
         <v>2410</v>
@@ -28813,6 +29121,9 @@
       <c r="U55" t="s">
         <v>135</v>
       </c>
+      <c r="V55" t="s">
+        <v>4490</v>
+      </c>
       <c r="W55" t="s">
         <v>2434</v>
       </c>
@@ -28882,8 +29193,14 @@
       <c r="AT55" t="s">
         <v>135</v>
       </c>
+      <c r="AU55" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV55" t="s">
         <v>135</v>
+      </c>
+      <c r="AW55" t="s">
+        <v>4490</v>
       </c>
       <c r="AX55" t="s">
         <v>2443</v>
@@ -29085,6 +29402,9 @@
       <c r="U56" t="s">
         <v>135</v>
       </c>
+      <c r="V56" t="s">
+        <v>4490</v>
+      </c>
       <c r="W56" t="s">
         <v>2465</v>
       </c>
@@ -29154,8 +29474,14 @@
       <c r="AT56" t="s">
         <v>135</v>
       </c>
+      <c r="AU56" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV56" t="s">
         <v>135</v>
+      </c>
+      <c r="AW56" t="s">
+        <v>4490</v>
       </c>
       <c r="AX56" t="s">
         <v>2475</v>
@@ -29429,8 +29755,14 @@
       <c r="AT57" t="s">
         <v>135</v>
       </c>
+      <c r="AU57" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV57" t="s">
         <v>135</v>
+      </c>
+      <c r="AW57" t="s">
+        <v>4490</v>
       </c>
       <c r="AX57" t="s">
         <v>2515</v>
@@ -29632,6 +29964,9 @@
       <c r="U58" t="s">
         <v>135</v>
       </c>
+      <c r="V58" t="s">
+        <v>4490</v>
+      </c>
       <c r="W58" t="s">
         <v>2546</v>
       </c>
@@ -29703,6 +30038,9 @@
       </c>
       <c r="AT58" t="s">
         <v>135</v>
+      </c>
+      <c r="AU58" t="s">
+        <v>4490</v>
       </c>
       <c r="AV58" t="s">
         <v>193</v>
@@ -29991,6 +30329,9 @@
       <c r="AV59" t="s">
         <v>135</v>
       </c>
+      <c r="AW59" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX59" t="s">
         <v>2599</v>
       </c>
@@ -30272,6 +30613,9 @@
       <c r="AV60" t="s">
         <v>135</v>
       </c>
+      <c r="AW60" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX60" t="s">
         <v>2636</v>
       </c>
@@ -30328,6 +30672,9 @@
       </c>
       <c r="BP60" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ60" t="s">
+        <v>128</v>
       </c>
       <c r="BR60" t="s">
         <v>108</v>
@@ -30466,6 +30813,9 @@
       <c r="U61" t="s">
         <v>135</v>
       </c>
+      <c r="V61" t="s">
+        <v>4490</v>
+      </c>
       <c r="W61" t="s">
         <v>2658</v>
       </c>
@@ -30535,9 +30885,15 @@
       <c r="AT61" t="s">
         <v>135</v>
       </c>
+      <c r="AU61" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV61" t="s">
         <v>135</v>
       </c>
+      <c r="AW61" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX61" t="s">
         <v>2666</v>
       </c>
@@ -30591,6 +30947,9 @@
       </c>
       <c r="BP61" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ61" t="s">
+        <v>128</v>
       </c>
       <c r="BR61" t="s">
         <v>108</v>
@@ -30801,8 +31160,14 @@
       <c r="AT62" t="s">
         <v>135</v>
       </c>
+      <c r="AU62" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV62" t="s">
         <v>135</v>
+      </c>
+      <c r="AW62" t="s">
+        <v>4490</v>
       </c>
       <c r="AX62" t="s">
         <v>2698</v>
@@ -31082,6 +31447,9 @@
       <c r="AV63" t="s">
         <v>135</v>
       </c>
+      <c r="AW63" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX63" t="s">
         <v>2736</v>
       </c>
@@ -31135,6 +31503,9 @@
       </c>
       <c r="BP63" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ63" t="s">
+        <v>128</v>
       </c>
       <c r="BR63" t="s">
         <v>108</v>
@@ -31354,6 +31725,9 @@
       <c r="AV64" t="s">
         <v>135</v>
       </c>
+      <c r="AW64" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX64" t="s">
         <v>371</v>
       </c>
@@ -31557,6 +31931,9 @@
       <c r="U65" t="s">
         <v>135</v>
       </c>
+      <c r="V65" t="s">
+        <v>4490</v>
+      </c>
       <c r="W65" t="s">
         <v>2799</v>
       </c>
@@ -31622,6 +31999,9 @@
       </c>
       <c r="AT65" t="s">
         <v>135</v>
+      </c>
+      <c r="AU65" t="s">
+        <v>4490</v>
       </c>
       <c r="AV65" t="s">
         <v>2810</v>
@@ -31829,6 +32209,9 @@
       <c r="U66" t="s">
         <v>135</v>
       </c>
+      <c r="V66" t="s">
+        <v>4490</v>
+      </c>
       <c r="W66" t="s">
         <v>2837</v>
       </c>
@@ -31898,6 +32281,9 @@
       <c r="AT66" t="s">
         <v>135</v>
       </c>
+      <c r="AU66" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV66" t="s">
         <v>193</v>
       </c>
@@ -31960,6 +32346,9 @@
       </c>
       <c r="BP66" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ66" t="s">
+        <v>128</v>
       </c>
       <c r="BR66" t="s">
         <v>108</v>
@@ -32104,6 +32493,9 @@
       <c r="U67" t="s">
         <v>135</v>
       </c>
+      <c r="V67" t="s">
+        <v>4490</v>
+      </c>
       <c r="W67" t="s">
         <v>2869</v>
       </c>
@@ -32460,6 +32852,9 @@
       <c r="AV68" t="s">
         <v>135</v>
       </c>
+      <c r="AW68" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX68" t="s">
         <v>371</v>
       </c>
@@ -32729,9 +33124,15 @@
       <c r="AT69" t="s">
         <v>135</v>
       </c>
+      <c r="AU69" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV69" t="s">
         <v>135</v>
       </c>
+      <c r="AW69" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX69" t="s">
         <v>136</v>
       </c>
@@ -32785,6 +33186,9 @@
       </c>
       <c r="BP69" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ69" t="s">
+        <v>128</v>
       </c>
       <c r="BR69" t="s">
         <v>108</v>
@@ -33007,6 +33411,9 @@
       <c r="AV70" t="s">
         <v>135</v>
       </c>
+      <c r="AW70" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX70" t="s">
         <v>2968</v>
       </c>
@@ -33060,6 +33467,9 @@
       </c>
       <c r="BP70" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ70" t="s">
+        <v>128</v>
       </c>
       <c r="BR70" t="s">
         <v>108</v>
@@ -33204,6 +33614,9 @@
       <c r="U71" t="s">
         <v>135</v>
       </c>
+      <c r="V71" t="s">
+        <v>4490</v>
+      </c>
       <c r="W71" t="s">
         <v>2989</v>
       </c>
@@ -33272,6 +33685,9 @@
       </c>
       <c r="AT71" t="s">
         <v>135</v>
+      </c>
+      <c r="AU71" t="s">
+        <v>4490</v>
       </c>
       <c r="AV71" t="s">
         <v>193</v>
@@ -33479,6 +33895,9 @@
       <c r="U72" t="s">
         <v>135</v>
       </c>
+      <c r="V72" t="s">
+        <v>4490</v>
+      </c>
       <c r="W72" t="s">
         <v>3016</v>
       </c>
@@ -33754,6 +34173,9 @@
       <c r="U73" t="s">
         <v>135</v>
       </c>
+      <c r="V73" t="s">
+        <v>4490</v>
+      </c>
       <c r="W73" t="s">
         <v>3051</v>
       </c>
@@ -33829,6 +34251,9 @@
       <c r="AV73" t="s">
         <v>135</v>
       </c>
+      <c r="AW73" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX73" t="s">
         <v>3060</v>
       </c>
@@ -33882,6 +34307,9 @@
       </c>
       <c r="BP73" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ73" t="s">
+        <v>128</v>
       </c>
       <c r="BR73" t="s">
         <v>108</v>
@@ -34026,6 +34454,9 @@
       <c r="U74" t="s">
         <v>135</v>
       </c>
+      <c r="V74" t="s">
+        <v>4490</v>
+      </c>
       <c r="W74" t="s">
         <v>3084</v>
       </c>
@@ -34100,6 +34531,9 @@
       </c>
       <c r="AV74" t="s">
         <v>135</v>
+      </c>
+      <c r="AW74" t="s">
+        <v>4490</v>
       </c>
       <c r="AX74" t="s">
         <v>3094</v>
@@ -34304,6 +34738,9 @@
       <c r="U75" t="s">
         <v>135</v>
       </c>
+      <c r="V75" t="s">
+        <v>4490</v>
+      </c>
       <c r="W75" t="s">
         <v>3121</v>
       </c>
@@ -34373,8 +34810,14 @@
       <c r="AT75" t="s">
         <v>135</v>
       </c>
+      <c r="AU75" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV75" t="s">
         <v>135</v>
+      </c>
+      <c r="AW75" t="s">
+        <v>4490</v>
       </c>
       <c r="AX75" t="s">
         <v>3127</v>
@@ -35213,8 +35656,14 @@
       <c r="AT78" t="s">
         <v>135</v>
       </c>
+      <c r="AU78" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV78" t="s">
         <v>135</v>
+      </c>
+      <c r="AW78" t="s">
+        <v>4490</v>
       </c>
       <c r="AX78" t="s">
         <v>3234</v>
@@ -35416,6 +35865,9 @@
       <c r="U79" t="s">
         <v>135</v>
       </c>
+      <c r="V79" t="s">
+        <v>4490</v>
+      </c>
       <c r="W79" t="s">
         <v>1533</v>
       </c>
@@ -35694,6 +36146,9 @@
       <c r="U80" t="s">
         <v>135</v>
       </c>
+      <c r="V80" t="s">
+        <v>4490</v>
+      </c>
       <c r="W80" t="s">
         <v>3294</v>
       </c>
@@ -35760,8 +36215,14 @@
       <c r="AT80" t="s">
         <v>135</v>
       </c>
+      <c r="AU80" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV80" t="s">
         <v>3300</v>
+      </c>
+      <c r="AW80" t="s">
+        <v>4490</v>
       </c>
       <c r="AX80" t="s">
         <v>3301</v>
@@ -35948,6 +36409,9 @@
       <c r="U81" t="s">
         <v>135</v>
       </c>
+      <c r="V81" t="s">
+        <v>4490</v>
+      </c>
       <c r="W81" t="s">
         <v>3322</v>
       </c>
@@ -36022,6 +36486,9 @@
       </c>
       <c r="AV81" t="s">
         <v>135</v>
+      </c>
+      <c r="AW81" t="s">
+        <v>4490</v>
       </c>
       <c r="AX81" t="s">
         <v>371</v>
@@ -36510,6 +36977,9 @@
       <c r="U83" t="s">
         <v>135</v>
       </c>
+      <c r="V83" t="s">
+        <v>4490</v>
+      </c>
       <c r="W83" t="s">
         <v>3404</v>
       </c>
@@ -36584,6 +37054,9 @@
       </c>
       <c r="AV83" t="s">
         <v>135</v>
+      </c>
+      <c r="AW83" t="s">
+        <v>4490</v>
       </c>
       <c r="AX83" t="s">
         <v>3411</v>
@@ -36920,6 +37393,9 @@
       <c r="BP84" t="s">
         <v>135</v>
       </c>
+      <c r="BQ84" t="s">
+        <v>128</v>
+      </c>
       <c r="BR84" t="s">
         <v>108</v>
       </c>
@@ -37063,6 +37539,9 @@
       <c r="U85" t="s">
         <v>135</v>
       </c>
+      <c r="V85" t="s">
+        <v>4490</v>
+      </c>
       <c r="W85" t="s">
         <v>3227</v>
       </c>
@@ -37132,6 +37611,9 @@
       <c r="AT85" t="s">
         <v>135</v>
       </c>
+      <c r="AU85" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV85" t="s">
         <v>193</v>
       </c>
@@ -37191,6 +37673,9 @@
       </c>
       <c r="BP85" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ85" t="s">
+        <v>128</v>
       </c>
       <c r="BR85" t="s">
         <v>108</v>
@@ -37326,6 +37811,9 @@
       <c r="U86" t="s">
         <v>135</v>
       </c>
+      <c r="V86" t="s">
+        <v>4490</v>
+      </c>
       <c r="W86" t="s">
         <v>3491</v>
       </c>
@@ -37394,6 +37882,9 @@
       </c>
       <c r="AT86" t="s">
         <v>135</v>
+      </c>
+      <c r="AU86" t="s">
+        <v>4490</v>
       </c>
       <c r="AV86" t="s">
         <v>193</v>
@@ -37679,6 +38170,9 @@
       <c r="AV87" t="s">
         <v>135</v>
       </c>
+      <c r="AW87" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX87" t="s">
         <v>371</v>
       </c>
@@ -37957,6 +38451,9 @@
       <c r="AV88" t="s">
         <v>135</v>
       </c>
+      <c r="AW88" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX88" t="s">
         <v>371</v>
       </c>
@@ -38157,6 +38654,9 @@
       <c r="U89" t="s">
         <v>135</v>
       </c>
+      <c r="V89" t="s">
+        <v>4490</v>
+      </c>
       <c r="W89" t="s">
         <v>3574</v>
       </c>
@@ -38226,8 +38726,14 @@
       <c r="AT89" t="s">
         <v>135</v>
       </c>
+      <c r="AU89" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV89" t="s">
         <v>135</v>
+      </c>
+      <c r="AW89" t="s">
+        <v>4490</v>
       </c>
       <c r="AX89" t="s">
         <v>3579</v>
@@ -38426,6 +38932,9 @@
       <c r="U90" t="s">
         <v>135</v>
       </c>
+      <c r="V90" t="s">
+        <v>4490</v>
+      </c>
       <c r="W90" t="s">
         <v>3227</v>
       </c>
@@ -38495,8 +39004,14 @@
       <c r="AT90" t="s">
         <v>135</v>
       </c>
+      <c r="AU90" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV90" t="s">
         <v>135</v>
+      </c>
+      <c r="AW90" t="s">
+        <v>4490</v>
       </c>
       <c r="AX90" t="s">
         <v>3601</v>
@@ -38698,6 +39213,9 @@
       <c r="U91" t="s">
         <v>135</v>
       </c>
+      <c r="V91" t="s">
+        <v>4490</v>
+      </c>
       <c r="W91" t="s">
         <v>3623</v>
       </c>
@@ -39054,6 +39572,9 @@
       <c r="AT92" t="s">
         <v>135</v>
       </c>
+      <c r="AU92" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV92" t="s">
         <v>193</v>
       </c>
@@ -39819,6 +40340,9 @@
       <c r="U95" t="s">
         <v>135</v>
       </c>
+      <c r="V95" t="s">
+        <v>4490</v>
+      </c>
       <c r="W95" t="s">
         <v>3227</v>
       </c>
@@ -39891,8 +40415,14 @@
       <c r="AT95" t="s">
         <v>135</v>
       </c>
+      <c r="AU95" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV95" t="s">
         <v>135</v>
+      </c>
+      <c r="AW95" t="s">
+        <v>4490</v>
       </c>
       <c r="AX95" t="s">
         <v>3759</v>
@@ -40094,6 +40624,9 @@
       <c r="U96" t="s">
         <v>135</v>
       </c>
+      <c r="V96" t="s">
+        <v>4490</v>
+      </c>
       <c r="W96" t="s">
         <v>3783</v>
       </c>
@@ -40168,6 +40701,9 @@
       </c>
       <c r="AV96" t="s">
         <v>135</v>
+      </c>
+      <c r="AW96" t="s">
+        <v>4490</v>
       </c>
       <c r="AX96" t="s">
         <v>3794</v>
@@ -40369,6 +40905,9 @@
       <c r="U97" t="s">
         <v>135</v>
       </c>
+      <c r="V97" t="s">
+        <v>4490</v>
+      </c>
       <c r="W97" t="s">
         <v>3824</v>
       </c>
@@ -40438,8 +40977,14 @@
       <c r="AT97" t="s">
         <v>135</v>
       </c>
+      <c r="AU97" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV97" t="s">
         <v>135</v>
+      </c>
+      <c r="AW97" t="s">
+        <v>4490</v>
       </c>
       <c r="AX97" t="s">
         <v>3833</v>
@@ -40722,6 +41267,9 @@
       <c r="AV98" t="s">
         <v>135</v>
       </c>
+      <c r="AW98" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX98" t="s">
         <v>3885</v>
       </c>
@@ -40919,6 +41467,9 @@
       <c r="U99" t="s">
         <v>135</v>
       </c>
+      <c r="V99" t="s">
+        <v>4490</v>
+      </c>
       <c r="W99" t="s">
         <v>3824</v>
       </c>
@@ -40988,9 +41539,15 @@
       <c r="AT99" t="s">
         <v>135</v>
       </c>
+      <c r="AU99" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV99" t="s">
         <v>135</v>
       </c>
+      <c r="AW99" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX99" t="s">
         <v>3925</v>
       </c>
@@ -41044,6 +41601,9 @@
       </c>
       <c r="BP99" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ99" t="s">
+        <v>128</v>
       </c>
       <c r="BR99" t="s">
         <v>108</v>
@@ -41188,6 +41748,9 @@
       <c r="U100" t="s">
         <v>135</v>
       </c>
+      <c r="V100" t="s">
+        <v>4490</v>
+      </c>
       <c r="W100" t="s">
         <v>3952</v>
       </c>
@@ -41466,6 +42029,9 @@
       <c r="U101" t="s">
         <v>135</v>
       </c>
+      <c r="V101" t="s">
+        <v>4490</v>
+      </c>
       <c r="W101" t="s">
         <v>4000</v>
       </c>
@@ -41538,8 +42104,14 @@
       <c r="AT101" t="s">
         <v>135</v>
       </c>
+      <c r="AU101" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV101" t="s">
         <v>135</v>
+      </c>
+      <c r="AW101" t="s">
+        <v>4490</v>
       </c>
       <c r="AX101" t="s">
         <v>4011</v>
@@ -42016,6 +42588,9 @@
       <c r="U103" t="s">
         <v>135</v>
       </c>
+      <c r="V103" t="s">
+        <v>4490</v>
+      </c>
       <c r="W103" t="s">
         <v>4081</v>
       </c>
@@ -42375,6 +42950,9 @@
       <c r="AV104" t="s">
         <v>135</v>
       </c>
+      <c r="AW104" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX104" t="s">
         <v>371</v>
       </c>
@@ -42569,6 +43147,9 @@
       <c r="U105" t="s">
         <v>135</v>
       </c>
+      <c r="V105" t="s">
+        <v>4490</v>
+      </c>
       <c r="W105" t="s">
         <v>4190</v>
       </c>
@@ -42646,6 +43227,9 @@
       </c>
       <c r="AV105" t="s">
         <v>135</v>
+      </c>
+      <c r="AW105" t="s">
+        <v>4490</v>
       </c>
       <c r="AX105" t="s">
         <v>4207</v>
@@ -42922,6 +43506,9 @@
       <c r="AV106" t="s">
         <v>135</v>
       </c>
+      <c r="AW106" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX106" t="s">
         <v>4258</v>
       </c>
@@ -42975,6 +43562,9 @@
       </c>
       <c r="BP106" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ106" t="s">
+        <v>128</v>
       </c>
       <c r="BR106" t="s">
         <v>108</v>
@@ -43113,6 +43703,9 @@
       <c r="U107" t="s">
         <v>135</v>
       </c>
+      <c r="V107" t="s">
+        <v>4490</v>
+      </c>
       <c r="W107" t="s">
         <v>4283</v>
       </c>
@@ -43182,9 +43775,15 @@
       <c r="AT107" t="s">
         <v>135</v>
       </c>
+      <c r="AU107" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV107" t="s">
         <v>135</v>
       </c>
+      <c r="AW107" t="s">
+        <v>4490</v>
+      </c>
       <c r="AX107" t="s">
         <v>136</v>
       </c>
@@ -43238,6 +43837,9 @@
       </c>
       <c r="BP107" t="s">
         <v>135</v>
+      </c>
+      <c r="BQ107" t="s">
+        <v>128</v>
       </c>
       <c r="BR107" t="s">
         <v>108</v>
@@ -43376,6 +43978,9 @@
       <c r="U108" t="s">
         <v>135</v>
       </c>
+      <c r="V108" t="s">
+        <v>4490</v>
+      </c>
       <c r="W108" t="s">
         <v>4320</v>
       </c>
@@ -43654,6 +44259,9 @@
       <c r="U109" t="s">
         <v>135</v>
       </c>
+      <c r="V109" t="s">
+        <v>4490</v>
+      </c>
       <c r="W109" t="s">
         <v>4361</v>
       </c>
@@ -43723,8 +44331,14 @@
       <c r="AT109" t="s">
         <v>135</v>
       </c>
+      <c r="AU109" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV109" t="s">
         <v>135</v>
+      </c>
+      <c r="AW109" t="s">
+        <v>4490</v>
       </c>
       <c r="AX109" t="s">
         <v>4370</v>
@@ -43998,8 +44612,14 @@
       <c r="AT110" t="s">
         <v>135</v>
       </c>
+      <c r="AU110" t="s">
+        <v>4490</v>
+      </c>
       <c r="AV110" t="s">
         <v>135</v>
+      </c>
+      <c r="AW110" t="s">
+        <v>4490</v>
       </c>
       <c r="AX110" t="s">
         <v>4412</v>
@@ -44200,6 +44820,9 @@
       </c>
       <c r="U111" t="s">
         <v>135</v>
+      </c>
+      <c r="V111" t="s">
+        <v>4490</v>
       </c>
       <c r="W111" t="s">
         <v>4442</v>

</xml_diff>